<commit_message>
feat(schema): move to OSCAL 1.2.3 and hold each enum to its metaschema list
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/oscal.xlsx
+++ b/project/excel/oscal.xlsx
@@ -2162,7 +2162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2188,50 +2188,60 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>props</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>links</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>date-authorized</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>security-sensitivity-level</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>system-information</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>security-impact-level</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>system-status</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>authorization-boundary</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>network-architecture</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>data-flow</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>responsible-parties</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>remarks</t>
         </is>

</xml_diff>

<commit_message>
fix(schema): name OSCAL's class key class_ so its page builds
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/oscal.xlsx
+++ b/project/excel/oscal.xlsx
@@ -736,7 +736,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -3393,7 +3393,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -3452,7 +3452,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -5266,7 +5266,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -5907,7 +5907,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -6353,7 +6353,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -6404,7 +6404,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -6584,7 +6584,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -6924,7 +6924,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -6980,7 +6980,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -7072,7 +7072,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -7296,7 +7296,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -8755,7 +8755,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -8816,7 +8816,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -8882,7 +8882,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>class_</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">

</xml_diff>

<commit_message>
chore(deps): move linkml and linkml-runtime to 1.12.1
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/oscal.xlsx
+++ b/project/excel/oscal.xlsx
@@ -166,15 +166,15 @@
     <sheet name="SspDiagramLink" sheetId="157" state="visible" r:id="rId157"/>
     <sheet name="SspLeveragedAuthorizationLink" sheetId="158" state="visible" r:id="rId158"/>
     <sheet name="SspByComponentLink" sheetId="159" state="visible" r:id="rId159"/>
-    <sheet name="SspSystemCharacteristicsResponsibleParty" sheetId="160" state="visible" r:id="rId160"/>
-    <sheet name="SspImplementedRequirementResponsibleRole" sheetId="161" state="visible" r:id="rId161"/>
+    <sheet name="SspSystemCharacteristics_d5c28d" sheetId="160" state="visible" r:id="rId160"/>
+    <sheet name="SspImplementedRequiremen_fa0d32" sheetId="161" state="visible" r:id="rId161"/>
     <sheet name="SspByComponentResponsibleRole" sheetId="162" state="visible" r:id="rId162"/>
     <sheet name="SspSystemComponent" sheetId="163" state="visible" r:id="rId163"/>
     <sheet name="SspInventoryItem" sheetId="164" state="visible" r:id="rId164"/>
     <sheet name="AssessmentResultsDocument" sheetId="165" state="visible" r:id="rId165"/>
     <sheet name="AssessmentResults" sheetId="166" state="visible" r:id="rId166"/>
     <sheet name="ImportAssessmentPlan" sheetId="167" state="visible" r:id="rId167"/>
-    <sheet name="AssessmentResultsLocalDefinitions" sheetId="168" state="visible" r:id="rId168"/>
+    <sheet name="AssessmentResultsLocalDe_39116c" sheetId="168" state="visible" r:id="rId168"/>
     <sheet name="Result" sheetId="169" state="visible" r:id="rId169"/>
     <sheet name="ResultLocalDefinitions" sheetId="170" state="visible" r:id="rId170"/>
     <sheet name="Attestation" sheetId="171" state="visible" r:id="rId171"/>

</xml_diff>

<commit_message>
fix(schema): give three OSCAL types without a typeof one (#26)
* fix(schema): give the three OSCAL types without a typeof one

Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>

* chore(deps): move linkml and linkml-runtime to 1.12.1

Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>

---------

Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/oscal.xlsx
+++ b/project/excel/oscal.xlsx
@@ -166,15 +166,15 @@
     <sheet name="SspDiagramLink" sheetId="157" state="visible" r:id="rId157"/>
     <sheet name="SspLeveragedAuthorizationLink" sheetId="158" state="visible" r:id="rId158"/>
     <sheet name="SspByComponentLink" sheetId="159" state="visible" r:id="rId159"/>
-    <sheet name="SspSystemCharacteristicsResponsibleParty" sheetId="160" state="visible" r:id="rId160"/>
-    <sheet name="SspImplementedRequirementResponsibleRole" sheetId="161" state="visible" r:id="rId161"/>
+    <sheet name="SspSystemCharacteristics_d5c28d" sheetId="160" state="visible" r:id="rId160"/>
+    <sheet name="SspImplementedRequiremen_fa0d32" sheetId="161" state="visible" r:id="rId161"/>
     <sheet name="SspByComponentResponsibleRole" sheetId="162" state="visible" r:id="rId162"/>
     <sheet name="SspSystemComponent" sheetId="163" state="visible" r:id="rId163"/>
     <sheet name="SspInventoryItem" sheetId="164" state="visible" r:id="rId164"/>
     <sheet name="AssessmentResultsDocument" sheetId="165" state="visible" r:id="rId165"/>
     <sheet name="AssessmentResults" sheetId="166" state="visible" r:id="rId166"/>
     <sheet name="ImportAssessmentPlan" sheetId="167" state="visible" r:id="rId167"/>
-    <sheet name="AssessmentResultsLocalDefinitions" sheetId="168" state="visible" r:id="rId168"/>
+    <sheet name="AssessmentResultsLocalDe_39116c" sheetId="168" state="visible" r:id="rId168"/>
     <sheet name="Result" sheetId="169" state="visible" r:id="rId169"/>
     <sheet name="ResultLocalDefinitions" sheetId="170" state="visible" r:id="rId170"/>
     <sheet name="Attestation" sheetId="171" state="visible" r:id="rId171"/>

</xml_diff>